<commit_message>
chore: actualizar datos unificados
Generado automaticamente por merge_sheets.py
</commit_message>
<xml_diff>
--- a/transformacion/InformeInventario_Unificado.xlsx
+++ b/transformacion/InformeInventario_Unificado.xlsx
@@ -448,62 +448,62 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Inventario - Inicial</t>
+          <t>Inventario Inicial</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Entradas - Almacén</t>
+          <t>Entradas Almacén</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Entradas por - Traslados</t>
+          <t>Entradas por Traslados</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Reintegros - Obra</t>
+          <t>Reintegros Obra</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Salidas - Almacén</t>
+          <t>Salidas Almacén</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Salidas por - Traslados</t>
+          <t>Salidas por Traslados</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Devoluciones - Proveedor</t>
+          <t>Devoluciones Proveedor</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Devoluciones - Valor</t>
+          <t>Devoluciones Valor</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Ajustes - Inventario</t>
+          <t>Ajustes Inventario</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Salidas - Bodega</t>
+          <t>Salidas Bodega</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Entradas - Bodega</t>
+          <t>Entradas Bodega</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>Inventario - Final</t>
+          <t>Inventario Final</t>
         </is>
       </c>
     </row>

</xml_diff>